<commit_message>
Atualiza TTD com novos assuntos
</commit_message>
<xml_diff>
--- a/data/reference/registros_suspeitos.xlsx
+++ b/data/reference/registros_suspeitos.xlsx
@@ -1,15 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udesc-my.sharepoint.com/personal/06376528945_udesc_br/Documents/Arquivo Permanente/sri_udesc_cct/data/reference/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_023583FD4BEB4F04AB2D4CD27D6E13ED7978A60B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CC202C5-7E1C-4BE0-82A3-A95F81D475E0}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -703,8 +714,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -744,9 +755,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -765,13 +774,94 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{497758BD-E48F-4739-9ADB-ECA4F30BC351}" name="Tabela1" displayName="Tabela1" ref="A1:T35" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:T35" xr:uid="{497758BD-E48F-4739-9ADB-ECA4F30BC351}"/>
+  <tableColumns count="20">
+    <tableColumn id="1" xr3:uid="{0C8E898C-2249-456E-A98B-2A94A8D9881D}" name="id_sistema"/>
+    <tableColumn id="2" xr3:uid="{489F842C-9187-4ABD-BF34-F371B2C2CA3E}" name="tipo_atividade"/>
+    <tableColumn id="3" xr3:uid="{1E44B751-E315-4538-988E-DBE209FC5D22}" name="eixo_usuario"/>
+    <tableColumn id="4" xr3:uid="{1B37F66B-F4CB-468F-84EA-1BFC6ED947A7}" name="publico_alvo"/>
+    <tableColumn id="5" xr3:uid="{A56D35FC-9A25-41F7-875E-C72A91402EAD}" name="acao_principal"/>
+    <tableColumn id="6" xr3:uid="{A7E6348C-F683-42D1-BFE3-75C7716B6628}" name="tipo_documental"/>
+    <tableColumn id="7" xr3:uid="{165A34EE-1DE1-46A2-B388-06D15A30A2AD}" name="termo_preferido_oficial"/>
+    <tableColumn id="8" xr3:uid="{EE49856B-61E4-47B4-A0D2-BA5370136751}" name="termos_populares_sugeridos"/>
+    <tableColumn id="9" xr3:uid="{9B550133-CECA-466B-B30B-3DA74607EDFC}" name="pergunta_guia_usuario"/>
+    <tableColumn id="10" xr3:uid="{2EEDD120-5734-47DF-A89D-56FE4C87CE56}" name="assunto_tecnico"/>
+    <tableColumn id="11" xr3:uid="{4E2AE4DF-FB22-49B7-92FC-8A3BF4F98FB3}" name="funcao"/>
+    <tableColumn id="12" xr3:uid="{BB8B329A-CCD1-404C-8C2B-5C72AC93054A}" name="subfuncao"/>
+    <tableColumn id="13" xr3:uid="{2CBC97AA-E5E8-4E2C-ACD3-5ADAC66E9C77}" name="atividade"/>
+    <tableColumn id="14" xr3:uid="{490DF5B7-06E7-4E9C-9B1C-4AC8A2354307}" name="codigo_classificacao"/>
+    <tableColumn id="15" xr3:uid="{B01D1B63-ED19-4E6E-B36E-E46D14CCB8BB}" name="prazo_corrente"/>
+    <tableColumn id="16" xr3:uid="{FB824D4E-50FC-4AFF-BC96-FAE7D6B91FC3}" name="prazo_intermediario"/>
+    <tableColumn id="17" xr3:uid="{B294BEF6-65A3-46DC-800E-7040F7CBFE34}" name="destinacao"/>
+    <tableColumn id="18" xr3:uid="{9A18E081-E324-49F1-BB74-0A8ADBE38BF5}" name="observacao"/>
+    <tableColumn id="19" xr3:uid="{1818FC6B-AA3D-4B38-A4C3-727555253EDC}" name="texto_busca_sistema"/>
+    <tableColumn id="20" xr3:uid="{DA1A446E-0B51-44C2-B954-2FDC701B4B79}" name="confianca_revisao"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -813,7 +903,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -845,9 +935,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -879,6 +987,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1054,11 +1180,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T35"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="23.42578125" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" customWidth="1"/>
+    <col min="14" max="14" width="20.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16.5703125" customWidth="1"/>
+    <col min="16" max="16" width="21.28515625" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13.140625" customWidth="1"/>
+    <col min="19" max="19" width="21.7109375" customWidth="1"/>
+    <col min="20" max="20" width="19" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1267,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -1176,7 +1323,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1229,7 +1376,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1282,7 +1429,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1335,7 +1482,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="1:20">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1397,7 +1544,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="7" spans="1:20">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1456,7 +1603,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="8" spans="1:20">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1515,7 +1662,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="9" spans="1:20">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1574,7 +1721,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="10" spans="1:20">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1630,7 +1777,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="11" spans="1:20">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1686,7 +1833,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="12" spans="1:20">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1742,7 +1889,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="13" spans="1:20">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1801,7 +1948,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="14" spans="1:20">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1854,7 +2001,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="15" spans="1:20">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1910,7 +2057,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="16" spans="1:20">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -1969,7 +2116,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="17" spans="1:20">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -2028,7 +2175,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="18" spans="1:20">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -2084,7 +2231,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="19" spans="1:20">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -2143,7 +2290,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="20" spans="1:20">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -2202,7 +2349,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="21" spans="1:20">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -2258,7 +2405,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="22" spans="1:20">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -2314,7 +2461,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="23" spans="1:20">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -2370,7 +2517,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="24" spans="1:20">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -2426,7 +2573,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="25" spans="1:20">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -2485,7 +2632,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="26" spans="1:20">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>44</v>
       </c>
@@ -2544,7 +2691,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="27" spans="1:20">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>45</v>
       </c>
@@ -2597,7 +2744,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="28" spans="1:20">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>46</v>
       </c>
@@ -2653,7 +2800,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="29" spans="1:20">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -2706,7 +2853,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="30" spans="1:20">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -2762,7 +2909,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="31" spans="1:20">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>49</v>
       </c>
@@ -2818,7 +2965,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="32" spans="1:20">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -2871,7 +3018,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="33" spans="1:20">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>51</v>
       </c>
@@ -2927,7 +3074,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="34" spans="1:20">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>52</v>
       </c>
@@ -2983,7 +3130,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="35" spans="1:20">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>53</v>
       </c>
@@ -3044,5 +3191,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>